<commit_message>
Oppdater PM10 og NO2 døgnverdier for mars-mai og juni-august 2026
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Bystrategi_Grenland/Klima/Luftforurensing/PM10 og NO2 døgn mars-mai 2026.xlsx
+++ b/Data/Bystrategi_Grenland/Klima/Luftforurensing/PM10 og NO2 døgn mars-mai 2026.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{28373EBB-3F05-46B8-8A76-9C2E7C7D99F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C249BB82-D03B-4430-9CC8-F7962A2CB31B}"/>
   <bookViews>
-    <workbookView xWindow="19740" yWindow="0" windowWidth="37290" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="38610" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>